<commit_message>
Actualiza integración de país y análisis exploratorio
</commit_message>
<xml_diff>
--- a/processed/diccionario_variables.xlsx
+++ b/processed/diccionario_variables.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -640,10 +640,44 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Categoría temática asociada con la clasificación del indicador.</t>
+          <t>Categoría utilizada para organizar la descarga inicial del indicador: Environment, Social, Governance u Other</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Pais_sede</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>País donde se localiza la sede corporativa de la empresa evaluada o, cuando corresponde, de su empresa matriz.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Fuente_pais</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Enlace a la fuente utilizada para verificar el país de sede asignado a la empresa o a su empresa matriz.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>Texto</t>
         </is>

</xml_diff>